<commit_message>
Complete Phase A–E: wrong book, practice, exam, import, and settings polish.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/判断题.xlsx
+++ b/public/templates/判断题.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,6 +430,9 @@
       <c r="J1" t="str">
         <v>标签</v>
       </c>
+      <c r="K1" t="str">
+        <v>领域</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -462,10 +465,13 @@
       <c r="J2" t="str">
         <v>媒体</v>
       </c>
+      <c r="K2" t="str">
+        <v>媒体</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>